<commit_message>
Improved detecting answers in LLM responses in parse_answer() and iImproved prompting for smaller models
</commit_message>
<xml_diff>
--- a/math/Experiments/Qwen2.5_7b/experiment_results_qwen2.5_7b_improved.xlsx
+++ b/math/Experiments/Qwen2.5_7b/experiment_results_qwen2.5_7b_improved.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/89c2773904d5ab9b/Dokumenter/Datalogi/Semester 6/Bachelor/llm_multiagent_debate_cachesaver-1/math/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/89c2773904d5ab9b/Dokumenter/Datalogi/Semester 6/Bachelor/llm_multiagent_debate_cachesaver-1/math/Experiments/Qwen2.5_7b/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_2B59D2BFD3F0D84F9B393511594B107471EFED8F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6140C5F5-8AFF-43C4-A2EB-0115827D0A48}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="11_2B59D2BFD3F0D84F9B393511594B107471EFED8F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A62DD94C-2373-41BA-8622-845A042234B2}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="2196" yWindow="2196" windowWidth="17280" windowHeight="9708" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -159,6 +159,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1277,6 +1281,14 @@
         <f t="shared" si="0"/>
         <v>4392</v>
       </c>
+      <c r="H30">
+        <f>SUM(H2:H28)</f>
+        <v>26754</v>
+      </c>
+      <c r="I30">
+        <f t="shared" ref="I30" si="1">SUM(I2:I28)</f>
+        <v>1141.3300000000002</v>
+      </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="D31" t="s">
@@ -1287,12 +1299,20 @@
         <v>0.98777777777777787</v>
       </c>
       <c r="F31" s="2">
-        <f t="shared" ref="F31:G31" si="1">AVERAGE(F2:F28)</f>
+        <f t="shared" ref="F31:G31" si="2">AVERAGE(F2:F28)</f>
         <v>828.22222222222217</v>
       </c>
       <c r="G31" s="2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>162.66666666666666</v>
+      </c>
+      <c r="H31" s="2">
+        <f>AVERAGE(H2:H28)</f>
+        <v>990.88888888888891</v>
+      </c>
+      <c r="I31" s="2">
+        <f t="shared" ref="I31" si="3">AVERAGE(I2:I28)</f>
+        <v>42.271481481481487</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.3">

</xml_diff>